<commit_message>
Report: into a script
</commit_message>
<xml_diff>
--- a/report/by_model_ethics.xlsx
+++ b/report/by_model_ethics.xlsx
@@ -607,11 +607,11 @@
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>53.9% ± 3.2%</t>
+          <t>53.6% ± 2.9%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>62.5% ± 11.4%</t>
+          <t>62.0% ± 10.8%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -648,11 +648,11 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>52.7% ± 3.0%</t>
+          <t>52.5% ± 3.2%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>59.9% ± 10.4%</t>
+          <t>59.2% ± 11.0%</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -683,23 +683,27 @@
       <c r="C8" t="n">
         <v>355</v>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="E8" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>61.2% ± 11.0%</t>
+          <t>65.7% ± 10.1%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>73.3%</t>
+          <t>74.1%</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>71.3% ± 20.9%</t>
+          <t>79.0% ± 18.6%</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -720,32 +724,28 @@
       <c r="C9" t="n">
         <v>355</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>65.9% ± 10.5%</t>
+          <t>66.1% ± 10.8%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>74.1%</t>
+          <t>72.5%</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>78.6% ± 18.8%</t>
+          <t>80.6% ± 20.4%</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>91.3%</t>
+          <t>91.4%</t>
         </is>
       </c>
     </row>
@@ -761,28 +761,32 @@
       <c r="C10" t="n">
         <v>884</v>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="E10" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>54.3% ± 10.6%</t>
+          <t>59.5% ± 16.7%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>76.6%</t>
+          <t>78.8%</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>56.6% ± 13.2%</t>
+          <t>64.1% ± 24.4%</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>89.9%</t>
+          <t>92.3%</t>
         </is>
       </c>
     </row>
@@ -798,32 +802,28 @@
       <c r="C11" t="n">
         <v>884</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>59.5% ± 16.7%</t>
+          <t>51.8% ± 7.5%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>78.8%</t>
+          <t>70.8%</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>64.1% ± 24.4%</t>
+          <t>52.9% ± 6.5%</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>70.0%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CI 95 for figs
</commit_message>
<xml_diff>
--- a/report/by_model_ethics.xlsx
+++ b/report/by_model_ethics.xlsx
@@ -473,13 +473,13 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Commonsense Hard Set</t>
+          <t>Commonsense Hard Set, % ± STD</t>
         </is>
       </c>
       <c r="G1" s="1" t="n"/>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Commonsense Test Set</t>
+          <t>Commonsense Test Set, % ± STD</t>
         </is>
       </c>
       <c r="I1" s="1" t="n"/>
@@ -533,22 +533,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>47.3% ± 14.7%</t>
+          <t>47.3 ± 14.7</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>55.5%</t>
+          <t>55.5</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>57.0% ± 7.3%</t>
+          <t>57.0 ± 7.3</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>73.7%</t>
+          <t>73.7</t>
         </is>
       </c>
     </row>
@@ -574,22 +574,22 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>52.3% ± 2.3%</t>
+          <t>52.3 ± 2.3</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>55.4%</t>
+          <t>55.4</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>58.3% ± 8.8%</t>
+          <t>58.3 ± 8.8</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>71.7%</t>
+          <t>71.7</t>
         </is>
       </c>
     </row>
@@ -611,22 +611,22 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>53.6% ± 2.9%</t>
+          <t>53.6 ± 2.9</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>61.8%</t>
+          <t>61.8</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>62.0% ± 10.8%</t>
+          <t>62.0 ± 10.8</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>85.4%</t>
+          <t>85.4</t>
         </is>
       </c>
     </row>
@@ -652,22 +652,22 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>52.5% ± 3.2%</t>
+          <t>52.5 ± 3.2</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>58.8%</t>
+          <t>58.8</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>59.2% ± 11.0%</t>
+          <t>59.2 ± 11.0</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>79.3%</t>
+          <t>79.3</t>
         </is>
       </c>
     </row>
@@ -693,22 +693,22 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>65.7% ± 10.1%</t>
+          <t>65.7 ± 10.1</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>74.1%</t>
+          <t>74.1</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>79.0% ± 18.6%</t>
+          <t>79.0 ± 18.6</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>91.8%</t>
+          <t>91.8</t>
         </is>
       </c>
     </row>
@@ -730,22 +730,22 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>66.1% ± 10.8%</t>
+          <t>66.1 ± 10.8</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>72.5%</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>80.6% ± 20.4%</t>
+          <t>80.6 ± 20.4</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>91.4%</t>
+          <t>91.4</t>
         </is>
       </c>
     </row>
@@ -771,22 +771,22 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>59.5% ± 16.7%</t>
+          <t>59.5 ± 16.7</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>78.8%</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>64.1% ± 24.4%</t>
+          <t>64.1 ± 24.4</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>92.3</t>
         </is>
       </c>
     </row>
@@ -808,22 +808,22 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>51.8% ± 7.5%</t>
+          <t>51.8 ± 7.5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>70.8%</t>
+          <t>70.8</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>52.9% ± 6.5%</t>
+          <t>52.9 ± 6.5</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>70.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CI 95 for tables
</commit_message>
<xml_diff>
--- a/report/by_model_ethics.xlsx
+++ b/report/by_model_ethics.xlsx
@@ -473,13 +473,13 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Commonsense Hard Set, % ± STD</t>
+          <t>Commonsense Hard Set, % (95% CI)</t>
         </is>
       </c>
       <c r="G1" s="1" t="n"/>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Commonsense Test Set, % ± STD</t>
+          <t>Commonsense Test Set, % (95% CI)</t>
         </is>
       </c>
       <c r="I1" s="1" t="n"/>
@@ -533,7 +533,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>47.3 ± 14.7</t>
+          <t>47.3 (0.0, 53.9)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>57.0 ± 7.3</t>
+          <t>57.0 (48.8, 70.5)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>52.3 ± 2.3</t>
+          <t>52.3 (50.0, 55.3)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>58.3 ± 8.8</t>
+          <t>58.3 (50.0, 71.0)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>53.6 ± 2.9</t>
+          <t>53.6 (49.4, 59.0)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>62.0 ± 10.8</t>
+          <t>62.0 (48.5, 78.7)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>52.5 ± 3.2</t>
+          <t>52.5 (48.2, 58.8)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>59.2 ± 11.0</t>
+          <t>59.2 (43.9, 78.8)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>65.7 ± 10.1</t>
+          <t>65.7 (49.8, 73.8)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>79.0 ± 18.6</t>
+          <t>79.0 (49.7, 91.6)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>66.1 ± 10.8</t>
+          <t>66.1 (51.5, 72.4)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>80.6 ± 20.4</t>
+          <t>80.6 (53.0, 91.4)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>59.5 ± 16.7</t>
+          <t>59.5 (49.8, 77.4)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>64.1 ± 24.4</t>
+          <t>64.1 (49.9, 90.2)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>51.8 ± 7.5</t>
+          <t>51.8 (45.9, 67.4)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>52.9 ± 6.5</t>
+          <t>52.9 (49.9, 66.6)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">

</xml_diff>